<commit_message>
Momentum scan results 2026-10-13
</commit_message>
<xml_diff>
--- a/results/momentum_2026-10-13.xlsx
+++ b/results/momentum_2026-10-13.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,12 +441,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ECHO</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -456,137 +456,111 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>GOOGL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>OPCH</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>BORR</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>GTLB</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>PLTR</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PENG</t>
+          <t>IBRX</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>EBAY</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>PANW</t>
-        </is>
-      </c>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>GTLB</t>
+          <t>SUNB</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SHOP</t>
+          <t>LYFT</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>EXEL</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>TRMD</t>
-        </is>
-      </c>
+          <t>OPCH</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>MRNA</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SPCX</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>GMAB</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>VYLR</t>
-        </is>
-      </c>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>PTC</t>
+          <t>P</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FRSH</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>SUNB</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>OKTA</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>NTSK</t>
-        </is>
-      </c>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PLTR</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>TECH</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>AFRM</t>
-        </is>
-      </c>
+          <t>PENG</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>INTR</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>